<commit_message>
Updated *7th sem result
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Imp\Coding\Python\Projects\Selenium\RGPV Result Bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{72A5A024-5234-450E-ABBB-728D127096D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{37B24149-9C8F-42EF-A4FD-6A081DDB5D30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3DD17C25-E4F6-4485-8627-B91891F35C26}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F46D43C8-845A-45F9-8677-DAC23F551997}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="1" r:id="rId1"/>
@@ -20,9 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="157">
-  <si>
-    <t>Roll No.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="149">
+  <si>
+    <t>Roll_No</t>
   </si>
   <si>
     <t>Name</t>
@@ -37,16 +37,13 @@
     <t>CGPA</t>
   </si>
   <si>
-    <t>AL-501</t>
-  </si>
-  <si>
-    <t>AL-502</t>
-  </si>
-  <si>
-    <t>AL-503</t>
-  </si>
-  <si>
-    <t>AL-504</t>
+    <t>AL-701</t>
+  </si>
+  <si>
+    <t>AL-702</t>
+  </si>
+  <si>
+    <t>AL-703</t>
   </si>
   <si>
     <t>0827AL221080</t>
@@ -58,12 +55,12 @@
     <t>PASS</t>
   </si>
   <si>
+    <t>C+</t>
+  </si>
+  <si>
     <t>B</t>
   </si>
   <si>
-    <t>C+</t>
-  </si>
-  <si>
     <t>0827AL221081</t>
   </si>
   <si>
@@ -94,45 +91,39 @@
     <t>MRUNANK DEKHNE</t>
   </si>
   <si>
+    <t>0827AL221085</t>
+  </si>
+  <si>
+    <t>MUJIB SHEIKH</t>
+  </si>
+  <si>
+    <t>0827AL221086</t>
+  </si>
+  <si>
+    <t>MUSKAN PATEL</t>
+  </si>
+  <si>
+    <t>0827AL221087</t>
+  </si>
+  <si>
+    <t>NAIVEDHYA SHARMA</t>
+  </si>
+  <si>
+    <t>0827AL221088</t>
+  </si>
+  <si>
+    <t>NAMAN PARMAR</t>
+  </si>
+  <si>
     <t>D</t>
   </si>
   <si>
-    <t>0827AL221085</t>
-  </si>
-  <si>
-    <t>MUJIB SHEIKH</t>
-  </si>
-  <si>
-    <t>0827AL221086</t>
-  </si>
-  <si>
-    <t>MUSKAN PATEL</t>
-  </si>
-  <si>
-    <t>0827AL221087</t>
-  </si>
-  <si>
-    <t>NAIVEDHYA SHARMA</t>
-  </si>
-  <si>
-    <t>0827AL221088</t>
-  </si>
-  <si>
-    <t>NAMAN PARMAR</t>
-  </si>
-  <si>
     <t>0827AL221090</t>
   </si>
   <si>
     <t>NIKHIL MEENA</t>
   </si>
   <si>
-    <t>0827AL221091</t>
-  </si>
-  <si>
-    <t>NIKITA CHAVHAN</t>
-  </si>
-  <si>
     <t>0827AL221093</t>
   </si>
   <si>
@@ -145,12 +136,6 @@
     <t>PALAK YADAV</t>
   </si>
   <si>
-    <t>0827AL221095</t>
-  </si>
-  <si>
-    <t>PALASH JAIN</t>
-  </si>
-  <si>
     <t>0827AL221096</t>
   </si>
   <si>
@@ -223,6 +208,9 @@
     <t>RAJ YADAV</t>
   </si>
   <si>
+    <t>A</t>
+  </si>
+  <si>
     <t>0827AL221108</t>
   </si>
   <si>
@@ -367,6 +355,12 @@
     <t>SUJAL BANKER</t>
   </si>
   <si>
+    <t>0827AL221134</t>
+  </si>
+  <si>
+    <t>SUJAL CHAWADA</t>
+  </si>
+  <si>
     <t>0827AL221135</t>
   </si>
   <si>
@@ -421,12 +415,6 @@
     <t>VIDIT DUBEY</t>
   </si>
   <si>
-    <t>0827AL221145</t>
-  </si>
-  <si>
-    <t>VIDIT SHARMA</t>
-  </si>
-  <si>
     <t>0827AL221146</t>
   </si>
   <si>
@@ -445,34 +433,22 @@
     <t>VISHAL JAISWAL</t>
   </si>
   <si>
-    <t>0827AL221149</t>
-  </si>
-  <si>
-    <t>VIVEK ANAND</t>
-  </si>
-  <si>
     <t>0827AL221150</t>
   </si>
   <si>
     <t>YASH MISHRA</t>
   </si>
   <si>
-    <t>0827AL221151</t>
-  </si>
-  <si>
-    <t>YASH RAJ KURAWARE</t>
-  </si>
-  <si>
-    <t>0827AL221152</t>
-  </si>
-  <si>
-    <t>YASH SHARMA</t>
-  </si>
-  <si>
     <t>0827AL221153</t>
   </si>
   <si>
     <t>YASH THAKUR</t>
+  </si>
+  <si>
+    <t>Fail in AL702</t>
+  </si>
+  <si>
+    <t>F</t>
   </si>
   <si>
     <t>0827AL221154</t>
@@ -1350,11 +1326,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF585802-6EA5-446D-BB18-94DD5F94F7E1}">
-  <dimension ref="A1:I72"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D7C9CD3-BECB-45E7-AF43-D34AF1AB6819}">
+  <dimension ref="A1:H67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1379,707 +1359,632 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D2">
+        <v>8.0399999999999991</v>
+      </c>
+      <c r="E2">
+        <v>7.4</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <v>8.58</v>
+      </c>
+      <c r="E3">
+        <v>8.5399999999999991</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>8.17</v>
+      </c>
+      <c r="E4">
+        <v>7.46</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5">
         <v>7.38</v>
       </c>
-      <c r="E2">
-        <v>7.28</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="E5">
+        <v>6.91</v>
+      </c>
+      <c r="F5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>7.88</v>
+      </c>
+      <c r="E6">
+        <v>6.17</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7">
+        <v>7.75</v>
+      </c>
+      <c r="E7">
+        <v>6.84</v>
+      </c>
+      <c r="F7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8">
+        <v>7.88</v>
+      </c>
+      <c r="E8">
+        <v>6.82</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9">
+        <v>7.38</v>
+      </c>
+      <c r="E9">
+        <v>6.7</v>
+      </c>
+      <c r="F9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10">
+        <v>6.92</v>
+      </c>
+      <c r="E10">
+        <v>6.1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11">
+        <v>6.75</v>
+      </c>
+      <c r="E11">
+        <v>6.51</v>
+      </c>
+      <c r="F11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12">
+        <v>7.42</v>
+      </c>
+      <c r="E12">
+        <v>6.54</v>
+      </c>
+      <c r="F12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" t="s">
+        <v>20</v>
+      </c>
+      <c r="H12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13">
+        <v>8.1300000000000008</v>
+      </c>
+      <c r="E13">
+        <v>7.4</v>
+      </c>
+      <c r="F13" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H13" t="s">
         <v>15</v>
       </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3">
-        <v>8.92</v>
-      </c>
-      <c r="E3">
-        <v>8.4600000000000009</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4">
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14">
+        <v>7.42</v>
+      </c>
+      <c r="E14">
+        <v>6.89</v>
+      </c>
+      <c r="F14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15">
+        <v>7.21</v>
+      </c>
+      <c r="E15">
+        <v>6.5</v>
+      </c>
+      <c r="F15" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" t="s">
+        <v>20</v>
+      </c>
+      <c r="H15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16">
+        <v>7.88</v>
+      </c>
+      <c r="E16">
+        <v>7.32</v>
+      </c>
+      <c r="F16" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" t="s">
+        <v>11</v>
+      </c>
+      <c r="H16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17">
+        <v>8.2899999999999991</v>
+      </c>
+      <c r="E17">
+        <v>8.1</v>
+      </c>
+      <c r="F17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18">
+        <v>7.75</v>
+      </c>
+      <c r="E18">
+        <v>7.12</v>
+      </c>
+      <c r="F18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" t="s">
+        <v>11</v>
+      </c>
+      <c r="H18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19">
+        <v>7.5</v>
+      </c>
+      <c r="E19">
+        <v>6.35</v>
+      </c>
+      <c r="F19" t="s">
+        <v>20</v>
+      </c>
+      <c r="G19" t="s">
+        <v>11</v>
+      </c>
+      <c r="H19" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20">
         <v>7.63</v>
       </c>
-      <c r="E4">
-        <v>7.21</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="E20">
+        <v>6.71</v>
+      </c>
+      <c r="F20" t="s">
         <v>20</v>
       </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5">
-        <v>7.29</v>
-      </c>
-      <c r="E5">
-        <v>6.74</v>
-      </c>
-      <c r="F5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6">
-        <v>6.38</v>
-      </c>
-      <c r="E6">
-        <v>5.7</v>
-      </c>
-      <c r="F6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G6" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7">
-        <v>7.46</v>
-      </c>
-      <c r="E7">
-        <v>6.54</v>
-      </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8">
-        <v>7.5</v>
-      </c>
-      <c r="E8">
-        <v>6.46</v>
-      </c>
-      <c r="F8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" t="s">
-        <v>13</v>
-      </c>
-      <c r="I8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9">
-        <v>7</v>
-      </c>
-      <c r="E9">
-        <v>6.59</v>
-      </c>
-      <c r="F9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" t="s">
-        <v>13</v>
-      </c>
-      <c r="I9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10">
-        <v>6.71</v>
-      </c>
-      <c r="E10">
-        <v>5.85</v>
-      </c>
-      <c r="F10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" t="s">
-        <v>24</v>
-      </c>
-      <c r="I10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11">
-        <v>6.71</v>
-      </c>
-      <c r="E11">
-        <v>6.4</v>
-      </c>
-      <c r="F11" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H11" t="s">
-        <v>13</v>
-      </c>
-      <c r="I11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12">
-        <v>6.17</v>
-      </c>
-      <c r="E12">
-        <v>5.58</v>
-      </c>
-      <c r="F12" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" t="s">
-        <v>21</v>
-      </c>
-      <c r="I12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" t="s">
-        <v>38</v>
-      </c>
-      <c r="C13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13">
-        <v>7.29</v>
-      </c>
-      <c r="E13">
-        <v>6.21</v>
-      </c>
-      <c r="F13" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" t="s">
-        <v>12</v>
-      </c>
-      <c r="H13" t="s">
-        <v>12</v>
-      </c>
-      <c r="I13" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14">
-        <v>7.92</v>
-      </c>
-      <c r="E14">
-        <v>7.12</v>
-      </c>
-      <c r="F14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G14" t="s">
-        <v>12</v>
-      </c>
-      <c r="H14" t="s">
-        <v>12</v>
-      </c>
-      <c r="I14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15">
-        <v>8.2100000000000009</v>
-      </c>
-      <c r="E15">
-        <v>7</v>
-      </c>
-      <c r="F15" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" t="s">
-        <v>16</v>
-      </c>
-      <c r="H15" t="s">
-        <v>12</v>
-      </c>
-      <c r="I15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" t="s">
-        <v>44</v>
-      </c>
-      <c r="C16" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16">
-        <v>6.92</v>
-      </c>
-      <c r="E16">
-        <v>6.72</v>
-      </c>
-      <c r="F16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H16" t="s">
-        <v>13</v>
-      </c>
-      <c r="I16" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B17" t="s">
-        <v>46</v>
-      </c>
-      <c r="C17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17">
-        <v>6.67</v>
-      </c>
-      <c r="E17">
-        <v>6.28</v>
-      </c>
-      <c r="F17" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" t="s">
-        <v>21</v>
-      </c>
-      <c r="H17" t="s">
-        <v>21</v>
-      </c>
-      <c r="I17" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" t="s">
-        <v>48</v>
-      </c>
-      <c r="C18" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18">
-        <v>7.46</v>
-      </c>
-      <c r="E18">
-        <v>7.17</v>
-      </c>
-      <c r="F18" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" t="s">
-        <v>13</v>
-      </c>
-      <c r="H18" t="s">
-        <v>13</v>
-      </c>
-      <c r="I18" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B19" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19">
-        <v>8.67</v>
-      </c>
-      <c r="E19">
-        <v>8.02</v>
-      </c>
-      <c r="F19" t="s">
-        <v>16</v>
-      </c>
-      <c r="G19" t="s">
-        <v>16</v>
-      </c>
-      <c r="H19" t="s">
-        <v>16</v>
-      </c>
-      <c r="I19" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>51</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="G20" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>52</v>
       </c>
-      <c r="C20" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20">
-        <v>7</v>
-      </c>
-      <c r="E20">
-        <v>6.97</v>
-      </c>
-      <c r="F20" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" t="s">
-        <v>21</v>
-      </c>
-      <c r="H20" t="s">
-        <v>13</v>
-      </c>
-      <c r="I20" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="B21" t="s">
         <v>53</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21">
+        <v>7.63</v>
+      </c>
+      <c r="E21">
+        <v>6.7</v>
+      </c>
+      <c r="F21" t="s">
+        <v>20</v>
+      </c>
+      <c r="G21" t="s">
+        <v>11</v>
+      </c>
+      <c r="H21" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>54</v>
       </c>
-      <c r="C21" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21">
-        <v>6.67</v>
-      </c>
-      <c r="E21">
-        <v>6.03</v>
-      </c>
-      <c r="F21" t="s">
-        <v>21</v>
-      </c>
-      <c r="G21" t="s">
-        <v>24</v>
-      </c>
-      <c r="H21" t="s">
-        <v>21</v>
-      </c>
-      <c r="I21" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="B22" t="s">
         <v>55</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22">
+        <v>8.1300000000000008</v>
+      </c>
+      <c r="E22">
+        <v>7.35</v>
+      </c>
+      <c r="F22" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22" t="s">
+        <v>11</v>
+      </c>
+      <c r="H22" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>56</v>
       </c>
-      <c r="C22" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22">
-        <v>6.88</v>
-      </c>
-      <c r="E22">
-        <v>6.54</v>
-      </c>
-      <c r="F22" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" t="s">
-        <v>13</v>
-      </c>
-      <c r="H22" t="s">
-        <v>13</v>
-      </c>
-      <c r="I22" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="B23" t="s">
         <v>57</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23">
+        <v>7.88</v>
+      </c>
+      <c r="E23">
+        <v>7.15</v>
+      </c>
+      <c r="F23" t="s">
+        <v>11</v>
+      </c>
+      <c r="G23" t="s">
+        <v>20</v>
+      </c>
+      <c r="H23" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>58</v>
       </c>
-      <c r="C23" t="s">
-        <v>11</v>
-      </c>
-      <c r="D23">
-        <v>6.92</v>
-      </c>
-      <c r="E23">
-        <v>6.55</v>
-      </c>
-      <c r="F23" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" t="s">
-        <v>12</v>
-      </c>
-      <c r="H23" t="s">
-        <v>21</v>
-      </c>
-      <c r="I23" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
         <v>59</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24">
+        <v>8.1300000000000008</v>
+      </c>
+      <c r="E24">
+        <v>7.54</v>
+      </c>
+      <c r="F24" t="s">
+        <v>15</v>
+      </c>
+      <c r="G24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>60</v>
       </c>
-      <c r="C24" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24">
-        <v>7.96</v>
-      </c>
-      <c r="E24">
-        <v>7.05</v>
-      </c>
-      <c r="F24" t="s">
-        <v>16</v>
-      </c>
-      <c r="G24" t="s">
-        <v>16</v>
-      </c>
-      <c r="H24" t="s">
-        <v>12</v>
-      </c>
-      <c r="I24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="B25" t="s">
         <v>61</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25">
+        <v>8.3800000000000008</v>
+      </c>
+      <c r="E25">
+        <v>7.32</v>
+      </c>
+      <c r="F25" t="s">
+        <v>15</v>
+      </c>
+      <c r="G25" t="s">
+        <v>11</v>
+      </c>
+      <c r="H25" t="s">
         <v>62</v>
       </c>
-      <c r="C25" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25">
-        <v>7.33</v>
-      </c>
-      <c r="E25">
-        <v>6.91</v>
-      </c>
-      <c r="F25" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" t="s">
-        <v>13</v>
-      </c>
-      <c r="H25" t="s">
-        <v>13</v>
-      </c>
-      <c r="I25" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>63</v>
       </c>
@@ -2087,28 +1992,25 @@
         <v>64</v>
       </c>
       <c r="C26" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D26">
-        <v>7.5</v>
+        <v>7.75</v>
       </c>
       <c r="E26">
-        <v>7.47</v>
+        <v>6.93</v>
       </c>
       <c r="F26" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="G26" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H26" t="s">
-        <v>13</v>
-      </c>
-      <c r="I26" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>65</v>
       </c>
@@ -2116,28 +2018,25 @@
         <v>66</v>
       </c>
       <c r="C27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D27">
-        <v>7.67</v>
+        <v>7.92</v>
       </c>
       <c r="E27">
-        <v>6.97</v>
+        <v>7.57</v>
       </c>
       <c r="F27" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G27" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H27" t="s">
-        <v>13</v>
-      </c>
-      <c r="I27" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>67</v>
       </c>
@@ -2145,28 +2044,25 @@
         <v>68</v>
       </c>
       <c r="C28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D28">
-        <v>7.04</v>
+        <v>7.83</v>
       </c>
       <c r="E28">
-        <v>6.78</v>
+        <v>7.49</v>
       </c>
       <c r="F28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H28" t="s">
-        <v>21</v>
-      </c>
-      <c r="I28" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>69</v>
       </c>
@@ -2174,28 +2070,25 @@
         <v>70</v>
       </c>
       <c r="C29" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D29">
-        <v>8.08</v>
+        <v>6.46</v>
       </c>
       <c r="E29">
-        <v>7.46</v>
+        <v>5.71</v>
       </c>
       <c r="F29" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="G29" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="H29" t="s">
-        <v>13</v>
-      </c>
-      <c r="I29" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>71</v>
       </c>
@@ -2203,28 +2096,25 @@
         <v>72</v>
       </c>
       <c r="C30" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D30">
-        <v>8</v>
+        <v>8.2899999999999991</v>
       </c>
       <c r="E30">
-        <v>7.4</v>
+        <v>7.67</v>
       </c>
       <c r="F30" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H30" t="s">
-        <v>12</v>
-      </c>
-      <c r="I30" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>73</v>
       </c>
@@ -2232,28 +2122,25 @@
         <v>74</v>
       </c>
       <c r="C31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D31">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E31">
-        <v>5.57</v>
+        <v>6.4</v>
       </c>
       <c r="F31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G31" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="H31" t="s">
-        <v>21</v>
-      </c>
-      <c r="I31" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>75</v>
       </c>
@@ -2261,28 +2148,25 @@
         <v>76</v>
       </c>
       <c r="C32" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D32">
-        <v>8.3800000000000008</v>
+        <v>7.75</v>
       </c>
       <c r="E32">
-        <v>7.41</v>
+        <v>7.07</v>
       </c>
       <c r="F32" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G32" t="s">
         <v>12</v>
       </c>
       <c r="H32" t="s">
-        <v>16</v>
-      </c>
-      <c r="I32" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>77</v>
       </c>
@@ -2290,28 +2174,25 @@
         <v>78</v>
       </c>
       <c r="C33" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D33">
-        <v>6.96</v>
+        <v>6.63</v>
       </c>
       <c r="E33">
-        <v>6.26</v>
+        <v>5.85</v>
       </c>
       <c r="F33" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="G33" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H33" t="s">
-        <v>21</v>
-      </c>
-      <c r="I33" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>79</v>
       </c>
@@ -2319,28 +2200,25 @@
         <v>80</v>
       </c>
       <c r="C34" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D34">
+        <v>8.4600000000000009</v>
+      </c>
+      <c r="E34">
         <v>7.63</v>
       </c>
-      <c r="E34">
-        <v>6.89</v>
-      </c>
       <c r="F34" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H34" t="s">
-        <v>13</v>
-      </c>
-      <c r="I34" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>81</v>
       </c>
@@ -2348,28 +2226,25 @@
         <v>82</v>
       </c>
       <c r="C35" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D35">
-        <v>6.29</v>
+        <v>7.5</v>
       </c>
       <c r="E35">
-        <v>5.6</v>
+        <v>6.09</v>
       </c>
       <c r="F35" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H35" t="s">
-        <v>21</v>
-      </c>
-      <c r="I35" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>83</v>
       </c>
@@ -2377,13 +2252,13 @@
         <v>84</v>
       </c>
       <c r="C36" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D36">
-        <v>8.25</v>
+        <v>7.88</v>
       </c>
       <c r="E36">
-        <v>7.41</v>
+        <v>6.72</v>
       </c>
       <c r="F36" t="s">
         <v>12</v>
@@ -2392,13 +2267,10 @@
         <v>12</v>
       </c>
       <c r="H36" t="s">
-        <v>12</v>
-      </c>
-      <c r="I36" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>85</v>
       </c>
@@ -2406,28 +2278,25 @@
         <v>86</v>
       </c>
       <c r="C37" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D37">
-        <v>6.29</v>
+        <v>8.17</v>
       </c>
       <c r="E37">
-        <v>5.86</v>
+        <v>7.28</v>
       </c>
       <c r="F37" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H37" t="s">
-        <v>21</v>
-      </c>
-      <c r="I37" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>87</v>
       </c>
@@ -2435,28 +2304,25 @@
         <v>88</v>
       </c>
       <c r="C38" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D38">
-        <v>6.67</v>
+        <v>7.08</v>
       </c>
       <c r="E38">
-        <v>6.39</v>
+        <v>5.96</v>
       </c>
       <c r="F38" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="G38" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H38" t="s">
-        <v>13</v>
-      </c>
-      <c r="I38" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>89</v>
       </c>
@@ -2464,28 +2330,25 @@
         <v>90</v>
       </c>
       <c r="C39" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D39">
-        <v>7.79</v>
+        <v>7.63</v>
       </c>
       <c r="E39">
-        <v>7.1</v>
+        <v>6.93</v>
       </c>
       <c r="F39" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G39" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H39" t="s">
         <v>12</v>
       </c>
-      <c r="I39" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>91</v>
       </c>
@@ -2493,28 +2356,25 @@
         <v>92</v>
       </c>
       <c r="C40" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D40">
-        <v>5.88</v>
+        <v>8</v>
       </c>
       <c r="E40">
-        <v>5.71</v>
+        <v>6.74</v>
       </c>
       <c r="F40" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="G40" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H40" t="s">
-        <v>24</v>
-      </c>
-      <c r="I40" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>93</v>
       </c>
@@ -2522,28 +2382,25 @@
         <v>94</v>
       </c>
       <c r="C41" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D41">
-        <v>7.46</v>
+        <v>8.5399999999999991</v>
       </c>
       <c r="E41">
-        <v>6.69</v>
+        <v>7.57</v>
       </c>
       <c r="F41" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H41" t="s">
-        <v>13</v>
-      </c>
-      <c r="I41" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>95</v>
       </c>
@@ -2551,28 +2408,25 @@
         <v>96</v>
       </c>
       <c r="C42" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D42">
-        <v>7.38</v>
+        <v>8.2899999999999991</v>
       </c>
       <c r="E42">
-        <v>6.39</v>
+        <v>7.62</v>
       </c>
       <c r="F42" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G42" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="H42" t="s">
-        <v>13</v>
-      </c>
-      <c r="I42" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>97</v>
       </c>
@@ -2580,28 +2434,25 @@
         <v>98</v>
       </c>
       <c r="C43" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D43">
-        <v>7.96</v>
+        <v>8.0399999999999991</v>
       </c>
       <c r="E43">
-        <v>7.34</v>
+        <v>7.29</v>
       </c>
       <c r="F43" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="G43" t="s">
         <v>12</v>
       </c>
       <c r="H43" t="s">
-        <v>13</v>
-      </c>
-      <c r="I43" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>99</v>
       </c>
@@ -2609,28 +2460,25 @@
         <v>100</v>
       </c>
       <c r="C44" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D44">
-        <v>8.0399999999999991</v>
+        <v>7.63</v>
       </c>
       <c r="E44">
-        <v>7.41</v>
+        <v>6.92</v>
       </c>
       <c r="F44" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G44" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H44" t="s">
         <v>12</v>
       </c>
-      <c r="I44" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>101</v>
       </c>
@@ -2638,28 +2486,25 @@
         <v>102</v>
       </c>
       <c r="C45" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D45">
-        <v>8</v>
+        <v>7.71</v>
       </c>
       <c r="E45">
-        <v>7.15</v>
+        <v>6.5</v>
       </c>
       <c r="F45" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G45" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H45" t="s">
-        <v>12</v>
-      </c>
-      <c r="I45" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>103</v>
       </c>
@@ -2667,28 +2512,25 @@
         <v>104</v>
       </c>
       <c r="C46" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D46">
-        <v>7.79</v>
+        <v>8.33</v>
       </c>
       <c r="E46">
-        <v>6.59</v>
+        <v>7.5</v>
       </c>
       <c r="F46" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G46" t="s">
         <v>12</v>
       </c>
       <c r="H46" t="s">
-        <v>13</v>
-      </c>
-      <c r="I46" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>105</v>
       </c>
@@ -2696,28 +2538,25 @@
         <v>106</v>
       </c>
       <c r="C47" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D47">
-        <v>7.08</v>
+        <v>8.2899999999999991</v>
       </c>
       <c r="E47">
-        <v>6.1</v>
+        <v>7.43</v>
       </c>
       <c r="F47" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G47" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="H47" t="s">
-        <v>13</v>
-      </c>
-      <c r="I47" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>107</v>
       </c>
@@ -2725,13 +2564,13 @@
         <v>108</v>
       </c>
       <c r="C48" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D48">
         <v>8.17</v>
       </c>
       <c r="E48">
-        <v>7.21</v>
+        <v>7</v>
       </c>
       <c r="F48" t="s">
         <v>12</v>
@@ -2740,13 +2579,10 @@
         <v>12</v>
       </c>
       <c r="H48" t="s">
-        <v>13</v>
-      </c>
-      <c r="I48" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>109</v>
       </c>
@@ -2754,28 +2590,25 @@
         <v>110</v>
       </c>
       <c r="C49" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D49">
-        <v>8.2100000000000009</v>
+        <v>8.42</v>
       </c>
       <c r="E49">
-        <v>7.18</v>
+        <v>7.93</v>
       </c>
       <c r="F49" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G49" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="H49" t="s">
-        <v>12</v>
-      </c>
-      <c r="I49" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>111</v>
       </c>
@@ -2783,28 +2616,25 @@
         <v>112</v>
       </c>
       <c r="C50" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D50">
-        <v>7.42</v>
+        <v>7.88</v>
       </c>
       <c r="E50">
-        <v>6.54</v>
+        <v>6.81</v>
       </c>
       <c r="F50" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G50" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H50" t="s">
-        <v>13</v>
-      </c>
-      <c r="I50" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>113</v>
       </c>
@@ -2812,28 +2642,25 @@
         <v>114</v>
       </c>
       <c r="C51" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D51">
-        <v>8.25</v>
+        <v>8.7100000000000009</v>
       </c>
       <c r="E51">
-        <v>7.87</v>
+        <v>7.92</v>
       </c>
       <c r="F51" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G51" t="s">
         <v>12</v>
       </c>
       <c r="H51" t="s">
-        <v>12</v>
-      </c>
-      <c r="I51" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>115</v>
       </c>
@@ -2841,28 +2668,25 @@
         <v>116</v>
       </c>
       <c r="C52" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D52">
-        <v>8.5</v>
+        <v>8.17</v>
       </c>
       <c r="E52">
-        <v>7.73</v>
+        <v>6.83</v>
       </c>
       <c r="F52" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="G52" t="s">
         <v>12</v>
       </c>
       <c r="H52" t="s">
-        <v>16</v>
-      </c>
-      <c r="I52" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>117</v>
       </c>
@@ -2870,28 +2694,25 @@
         <v>118</v>
       </c>
       <c r="C53" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D53">
-        <v>7.67</v>
+        <v>8</v>
       </c>
       <c r="E53">
-        <v>6.47</v>
+        <v>6.82</v>
       </c>
       <c r="F53" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G53" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H53" t="s">
-        <v>12</v>
-      </c>
-      <c r="I53" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>119</v>
       </c>
@@ -2899,28 +2720,25 @@
         <v>120</v>
       </c>
       <c r="C54" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D54">
-        <v>7.25</v>
+        <v>8.17</v>
       </c>
       <c r="E54">
-        <v>6.55</v>
+        <v>7.07</v>
       </c>
       <c r="F54" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G54" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H54" t="s">
-        <v>13</v>
-      </c>
-      <c r="I54" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>121</v>
       </c>
@@ -2928,28 +2746,25 @@
         <v>122</v>
       </c>
       <c r="C55" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D55">
-        <v>7.46</v>
+        <v>7.71</v>
       </c>
       <c r="E55">
-        <v>6.73</v>
+        <v>6.21</v>
       </c>
       <c r="F55" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G55" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H55" t="s">
-        <v>13</v>
-      </c>
-      <c r="I55" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>123</v>
       </c>
@@ -2957,28 +2772,25 @@
         <v>124</v>
       </c>
       <c r="C56" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D56">
-        <v>5.88</v>
+        <v>8.5399999999999991</v>
       </c>
       <c r="E56">
-        <v>5.72</v>
+        <v>7.63</v>
       </c>
       <c r="F56" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G56" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H56" t="s">
-        <v>21</v>
-      </c>
-      <c r="I56" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>125</v>
       </c>
@@ -2986,28 +2798,25 @@
         <v>126</v>
       </c>
       <c r="C57" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D57">
-        <v>7.5</v>
+        <v>7.83</v>
       </c>
       <c r="E57">
-        <v>7.36</v>
+        <v>6.54</v>
       </c>
       <c r="F57" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G57" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H57" t="s">
-        <v>13</v>
-      </c>
-      <c r="I57" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>127</v>
       </c>
@@ -3015,28 +2824,25 @@
         <v>128</v>
       </c>
       <c r="C58" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D58">
-        <v>6.25</v>
+        <v>7.58</v>
       </c>
       <c r="E58">
-        <v>6.26</v>
+        <v>6.29</v>
       </c>
       <c r="F58" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G58" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="H58" t="s">
-        <v>21</v>
-      </c>
-      <c r="I58" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>129</v>
       </c>
@@ -3044,28 +2850,25 @@
         <v>130</v>
       </c>
       <c r="C59" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D59">
-        <v>5.92</v>
+        <v>8</v>
       </c>
       <c r="E59">
-        <v>6.04</v>
+        <v>7.06</v>
       </c>
       <c r="F59" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="G59" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="H59" t="s">
-        <v>21</v>
-      </c>
-      <c r="I59" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>131</v>
       </c>
@@ -3073,28 +2876,25 @@
         <v>132</v>
       </c>
       <c r="C60" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D60">
-        <v>7.58</v>
+        <v>8.2899999999999991</v>
       </c>
       <c r="E60">
-        <v>6.81</v>
+        <v>7.45</v>
       </c>
       <c r="F60" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G60" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H60" t="s">
-        <v>13</v>
-      </c>
-      <c r="I60" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>133</v>
       </c>
@@ -3102,28 +2902,25 @@
         <v>134</v>
       </c>
       <c r="C61" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D61">
-        <v>7.33</v>
+        <v>6.46</v>
       </c>
       <c r="E61">
-        <v>7.14</v>
+        <v>5.26</v>
       </c>
       <c r="F61" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="G61" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="H61" t="s">
-        <v>13</v>
-      </c>
-      <c r="I61" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>135</v>
       </c>
@@ -3131,28 +2928,25 @@
         <v>136</v>
       </c>
       <c r="C62" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D62">
-        <v>7.5</v>
+        <v>6.17</v>
       </c>
       <c r="E62">
-        <v>7.19</v>
+        <v>5.44</v>
       </c>
       <c r="F62" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="G62" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="H62" t="s">
-        <v>13</v>
-      </c>
-      <c r="I62" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>137</v>
       </c>
@@ -3160,28 +2954,25 @@
         <v>138</v>
       </c>
       <c r="C63" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D63">
-        <v>5.29</v>
+        <v>8.25</v>
       </c>
       <c r="E63">
-        <v>5.08</v>
+        <v>7.36</v>
       </c>
       <c r="F63" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="G63" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H63" t="s">
-        <v>21</v>
-      </c>
-      <c r="I63" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>139</v>
       </c>
@@ -3189,257 +2980,100 @@
         <v>140</v>
       </c>
       <c r="C64" t="s">
-        <v>11</v>
+        <v>141</v>
       </c>
       <c r="D64">
-        <v>5.33</v>
+        <v>5.79</v>
       </c>
       <c r="E64">
-        <v>5.22</v>
+        <v>5.61</v>
       </c>
       <c r="F64" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="G64" t="s">
-        <v>24</v>
+        <v>142</v>
       </c>
       <c r="H64" t="s">
-        <v>24</v>
-      </c>
-      <c r="I64" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B65" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C65" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D65">
-        <v>6.13</v>
+        <v>8.5399999999999991</v>
       </c>
       <c r="E65">
-        <v>6.06</v>
+        <v>8.31</v>
       </c>
       <c r="F65" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="G65" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="H65" t="s">
-        <v>21</v>
-      </c>
-      <c r="I65" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B66" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C66" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D66">
-        <v>7.92</v>
+        <v>8.42</v>
       </c>
       <c r="E66">
-        <v>7.13</v>
+        <v>8.23</v>
       </c>
       <c r="F66" t="s">
         <v>12</v>
       </c>
       <c r="G66" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H66" t="s">
-        <v>12</v>
-      </c>
-      <c r="I66" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B67" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C67" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D67">
-        <v>6.75</v>
+        <v>8.25</v>
       </c>
       <c r="E67">
-        <v>5.87</v>
+        <v>7.79</v>
       </c>
       <c r="F67" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="G67" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H67" t="s">
-        <v>21</v>
-      </c>
-      <c r="I67" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>147</v>
-      </c>
-      <c r="B68" t="s">
-        <v>148</v>
-      </c>
-      <c r="C68" t="s">
-        <v>11</v>
-      </c>
-      <c r="D68">
-        <v>7.13</v>
-      </c>
-      <c r="E68">
-        <v>6.99</v>
-      </c>
-      <c r="F68" t="s">
-        <v>12</v>
-      </c>
-      <c r="G68" t="s">
-        <v>21</v>
-      </c>
-      <c r="H68" t="s">
-        <v>21</v>
-      </c>
-      <c r="I68" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>149</v>
-      </c>
-      <c r="B69" t="s">
-        <v>150</v>
-      </c>
-      <c r="C69" t="s">
-        <v>11</v>
-      </c>
-      <c r="D69">
-        <v>5.21</v>
-      </c>
-      <c r="E69">
-        <v>5.45</v>
-      </c>
-      <c r="F69" t="s">
-        <v>21</v>
-      </c>
-      <c r="G69" t="s">
-        <v>21</v>
-      </c>
-      <c r="H69" t="s">
-        <v>24</v>
-      </c>
-      <c r="I69" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>151</v>
-      </c>
-      <c r="B70" t="s">
-        <v>152</v>
-      </c>
-      <c r="C70" t="s">
-        <v>11</v>
-      </c>
-      <c r="D70">
-        <v>8.6300000000000008</v>
-      </c>
-      <c r="E70">
-        <v>8.25</v>
-      </c>
-      <c r="F70" t="s">
-        <v>16</v>
-      </c>
-      <c r="G70" t="s">
-        <v>16</v>
-      </c>
-      <c r="H70" t="s">
-        <v>12</v>
-      </c>
-      <c r="I70" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>153</v>
-      </c>
-      <c r="B71" t="s">
-        <v>154</v>
-      </c>
-      <c r="C71" t="s">
-        <v>11</v>
-      </c>
-      <c r="D71">
-        <v>8.67</v>
-      </c>
-      <c r="E71">
-        <v>8.24</v>
-      </c>
-      <c r="F71" t="s">
-        <v>12</v>
-      </c>
-      <c r="G71" t="s">
-        <v>16</v>
-      </c>
-      <c r="H71" t="s">
-        <v>16</v>
-      </c>
-      <c r="I71" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>155</v>
-      </c>
-      <c r="B72" t="s">
-        <v>156</v>
-      </c>
-      <c r="C72" t="s">
-        <v>11</v>
-      </c>
-      <c r="D72">
-        <v>7.83</v>
-      </c>
-      <c r="E72">
-        <v>7.67</v>
-      </c>
-      <c r="F72" t="s">
-        <v>13</v>
-      </c>
-      <c r="G72" t="s">
-        <v>12</v>
-      </c>
-      <c r="H72" t="s">
-        <v>13</v>
-      </c>
-      <c r="I72" t="s">
-        <v>13</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>